<commit_message>
Lab 8 has been completed
</commit_message>
<xml_diff>
--- a/docs/Canonical/AlphaOmega/AlphaOmega Data Dictionary.xlsx
+++ b/docs/Canonical/AlphaOmega/AlphaOmega Data Dictionary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/70ee5aa1d6a4da1f/AlphaOmega/docs/Canonical/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CYRIL\docs\Canonical\AlphaOmega\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="190" documentId="8_{EEE9038B-07F8-4E74-ABBD-DCE8BEFA068C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F42C6716-8B22-44BF-9C7E-FD1FC863B6E9}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25E18AD3-B4FD-47E7-92D2-682604D29C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{2E56D5ED-1CE4-4881-8D7B-73E549022760}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{2E56D5ED-1CE4-4881-8D7B-73E549022760}"/>
   </bookViews>
   <sheets>
     <sheet name="Rules" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="sync_history" sheetId="6" r:id="rId6"/>
     <sheet name="source_containers" sheetId="7" r:id="rId7"/>
     <sheet name="sync_runs" sheetId="9" r:id="rId8"/>
+    <sheet name="scripts" sheetId="10" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">domains!$A$1:$F$1</definedName>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="221">
   <si>
     <t>Rule</t>
   </si>
@@ -775,6 +776,141 @@
       </rPr>
       <t>.</t>
     </r>
+  </si>
+  <si>
+    <t>Knowledge Object identity</t>
+  </si>
+  <si>
+    <t>A source object is identified by the unique combination of source_id and source_object_id. source_id alone and source_object_id alone are not sufficient.</t>
+  </si>
+  <si>
+    <t>Internal identifier for the script or SQL artifact record.</t>
+  </si>
+  <si>
+    <t>artifact_path</t>
+  </si>
+  <si>
+    <t>Repository-relative path identifying the documented artifact.</t>
+  </si>
+  <si>
+    <t>artifact_name</t>
+  </si>
+  <si>
+    <t>Artifact filename, including its extension.</t>
+  </si>
+  <si>
+    <t>artifact_type</t>
+  </si>
+  <si>
+    <t>Artifact classification, such as Python or SQL.</t>
+  </si>
+  <si>
+    <t>Plain-language statement of why the artifact exists.</t>
+  </si>
+  <si>
+    <t>responsibilities</t>
+  </si>
+  <si>
+    <t>Structured Metadata</t>
+  </si>
+  <si>
+    <t>List of responsibilities owned by the artifact.</t>
+  </si>
+  <si>
+    <t>exclusions</t>
+  </si>
+  <si>
+    <t>List of responsibilities explicitly outside the artifact’s scope.</t>
+  </si>
+  <si>
+    <t>classes</t>
+  </si>
+  <si>
+    <t>Classes defined by the artifact.</t>
+  </si>
+  <si>
+    <t>functions</t>
+  </si>
+  <si>
+    <t>Functions or methods defined by the artifact.</t>
+  </si>
+  <si>
+    <t>imports</t>
+  </si>
+  <si>
+    <t>Python modules or packages imported by the artifact.</t>
+  </si>
+  <si>
+    <t>referenced_tables</t>
+  </si>
+  <si>
+    <t>Database tables referenced by the artifact.</t>
+  </si>
+  <si>
+    <t>referenced_rpcs</t>
+  </si>
+  <si>
+    <t>Database remote procedures called by the artifact.</t>
+  </si>
+  <si>
+    <t>Hash of the scanned artifact content used to identify content changes between scans.</t>
+  </si>
+  <si>
+    <t>last_scanned_at</t>
+  </si>
+  <si>
+    <t>Most recent time the artifact metadata was scanned.</t>
+  </si>
+  <si>
+    <t>Indicates whether the artifact remains active in the current implementation.</t>
+  </si>
+  <si>
+    <t>module_docstring</t>
+  </si>
+  <si>
+    <t>Module-level documentation extracted from the artifact.</t>
+  </si>
+  <si>
+    <t>verifies</t>
+  </si>
+  <si>
+    <t>Behaviors or conditions verified by a test artifact.</t>
+  </si>
+  <si>
+    <t>referenced_scripts</t>
+  </si>
+  <si>
+    <t>Other repository scripts referenced by the artifact.</t>
+  </si>
+  <si>
+    <t>defined_rpcs</t>
+  </si>
+  <si>
+    <t>Database remote procedures defined by a SQL artifact.</t>
+  </si>
+  <si>
+    <t>line_count</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>integer</t>
+  </si>
+  <si>
+    <t>Number of lines in the scanned artifact.</t>
+  </si>
+  <si>
+    <t>scan_error</t>
+  </si>
+  <si>
+    <t>Error recorded when the documentation scan cannot fully process the artifact.</t>
+  </si>
+  <si>
+    <t>documentation_status</t>
+  </si>
+  <si>
+    <t>Documentation completeness status assigned by the artifact audit.</t>
   </si>
 </sst>
 </file>
@@ -892,16 +1028,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -911,6 +1038,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -926,10 +1060,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1249,28 +1379,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DB4BDDB-627A-41A5-BCC8-1AD09EEA205C}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22.140625" customWidth="1"/>
-    <col min="2" max="2" width="69.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="29" customWidth="1"/>
+    <col min="1" max="1" width="22.140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="69.85546875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="29" style="3" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" customHeight="1">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="D1" s="8"/>
-    </row>
-    <row r="2" spans="1:4" ht="30">
+      <c r="D1" s="13"/>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -1278,7 +1409,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="30">
+    <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -1326,60 +1457,68 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="60">
-      <c r="A9" s="10" t="s">
+    <row r="9" spans="1:4" ht="45">
+      <c r="A9" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="6" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="75">
-      <c r="A10" s="10" t="s">
+    <row r="10" spans="1:4" ht="60">
+      <c r="A10" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="6" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15" customHeight="1">
-      <c r="A11" s="10" t="s">
+    <row r="11" spans="1:4" ht="45">
+      <c r="A11" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="6" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="45">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="6" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="60">
-      <c r="A13" s="10" t="s">
+    <row r="13" spans="1:4" ht="45">
+      <c r="A13" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="6" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="45">
-      <c r="A14" s="10" t="s">
+    <row r="14" spans="1:4" ht="30">
+      <c r="A14" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="6" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="60">
-      <c r="A15" s="10" t="s">
+    <row r="15" spans="1:4" ht="45">
+      <c r="A15" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="6" t="s">
         <v>170</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="45">
+      <c r="A16" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2460,7 @@
       <c r="E6" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="8" t="s">
         <v>156</v>
       </c>
     </row>
@@ -2845,32 +2984,32 @@
       </c>
     </row>
     <row r="11" spans="1:6" ht="18">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="9" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="10" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="10" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="10" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="10" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="11" t="s">
         <v>148</v>
       </c>
     </row>
@@ -2991,38 +3130,516 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="18">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="9" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="10" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="10" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="10" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="13" t="s">
+      <c r="A11" s="10" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="10" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="10" t="s">
         <v>175</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2715954-4450-4E36-857E-1839C2B82682}">
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="77.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>220</v>
       </c>
     </row>
   </sheetData>

</xml_diff>